<commit_message>
feat: true up the accrual when the final invoice arrives
Once a platform media invoice covering the whole service month is
received (new is_media_final flag), it replaces the month-end estimate:
accrual 0 and recognised media expense = media invoiced, whether the
invoice came in above or below delivered spend. Before that the existing
estimate rule applies unchanged. Previously an invoice below delivered
spend left the difference accrued forever (Meta 2025-01: 27.30).

The identity test is renamed and derives finality independently; proven
by mutation (the old rule fails it on 12 rows). The Excel pack carries
the flag and applies the true-up in its formulas; samples recalculated
with all checks TRUE. Docs and worked example updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ccU24NxQXubfH6QKwwvw2
</commit_message>
<xml_diff>
--- a/reports/month_end/month_end_pack_2025-03.xlsx
+++ b/reports/month_end/month_end_pack_2025-03.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="114">
   <si>
     <t xml:space="preserve">Month-end marketing pack</t>
   </si>
@@ -104,16 +104,22 @@
     <t xml:space="preserve">Agency fee lines allocated to the channel (60/40 Meta/Google retainer). Not budgeted and not compared with delivered spend.</t>
   </si>
   <si>
+    <t xml:space="preserve">Final invoice received</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A platform media invoice covering the whole month has arrived. It then replaces the estimate: accrual 0, recognised media = media invoiced (the true-up).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Estimated unbilled accrual</t>
   </si>
   <si>
-    <t xml:space="preserve">MAX(delivered - media invoiced, 0): delivered media not yet invoiced.</t>
+    <t xml:space="preserve">Before the final invoice: MAX(delivered - media invoiced, 0), delivered media not yet invoiced. After it: 0.</t>
   </si>
   <si>
     <t xml:space="preserve">Recognised media expense</t>
   </si>
   <si>
-    <t xml:space="preserve">MAX(delivered, media invoiced). Blank delivered: media invoiced if any.</t>
+    <t xml:space="preserve">After the final invoice: media invoiced. Before it: MAX(delivered, media invoiced). Blank delivered: media invoiced if any.</t>
   </si>
   <si>
     <t xml:space="preserve">Recognised expense (incl. fees)</t>
@@ -203,6 +209,9 @@
     <t xml:space="preserve">data_status</t>
   </si>
   <si>
+    <t xml:space="preserve">is_media_final</t>
+  </si>
+  <si>
     <t xml:space="preserve">meta</t>
   </si>
   <si>
@@ -264,6 +273,9 @@
   </si>
   <si>
     <t xml:space="preserve">Budget with known spend (helper)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final invoice received (TRUE = true-up applied)</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -363,8 +375,8 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);\-"/>
-    <numFmt numFmtId="167" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);\-"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -509,7 +521,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -546,6 +558,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -570,23 +586,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -846,7 +866,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -1050,15 +1070,23 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
+      <c r="A28" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>45</v>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1077,62 +1105,65 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="1" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>11250</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>10804.33</v>
@@ -1159,21 +1190,25 @@
         <v>742.68</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>62</v>
+        <v>65</v>
+      </c>
+      <c r="N2" s="9" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>8500</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>8608.79</v>
@@ -1200,21 +1235,25 @@
         <v>28.4</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>65</v>
+        <v>68</v>
+      </c>
+      <c r="N3" s="9" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>1500</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="n">
@@ -1229,10 +1268,14 @@
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
       <c r="L4" s="7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>67</v>
+        <v>70</v>
+      </c>
+      <c r="N4" s="9" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1249,10 +1292,11 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>68</v>
+      <c r="A6" s="10" t="s">
+        <v>71</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1266,6 +1310,7 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
@@ -1283,6 +1328,7 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1300,16 +1346,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="2" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="2" style="0" width="17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1327,6 +1373,7 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -1348,16 +1395,17 @@
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -1373,12 +1421,13 @@
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="str">
+      <c r="B4" s="12" t="str">
         <f aca="false">'Read me'!B4</f>
         <v>2025-03</v>
       </c>
@@ -1397,12 +1446,13 @@
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" s="11" t="str">
+        <v>75</v>
+      </c>
+      <c r="B5" s="12" t="str">
         <f aca="false">'Read me'!B5</f>
         <v>2025-07-01</v>
       </c>
@@ -1421,6 +1471,7 @@
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
@@ -1440,110 +1491,114 @@
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="I7" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="J7" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="K7" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="L7" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="M7" s="12" t="s">
+      <c r="I7" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="N7" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="O7" s="12" t="s">
+      <c r="J7" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="K7" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="N7" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="P7" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q7" s="12" t="s">
-        <v>79</v>
+      <c r="O7" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="P7" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q7" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="R7" s="13" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="str">
+      <c r="A8" s="12" t="str">
         <f aca="false">Inputs!A2</f>
         <v>meta</v>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="14" t="n">
         <f aca="false">IF(Inputs!B2="","",Inputs!B2)</f>
         <v>11250</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <f aca="false">IF(Inputs!D2="","",Inputs!D2)</f>
         <v>10804.33</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <f aca="false">SUMIFS(Inputs!$E$2:$E$4,Inputs!$A$2:$A$4,$A8)</f>
         <v>11547.01</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="14" t="n">
         <f aca="false">SUMIFS(Inputs!$F$2:$F$4,Inputs!$A$2:$A$4,$A8)</f>
         <v>1700</v>
       </c>
-      <c r="F8" s="14" t="n">
-        <f aca="false">IF(C8="","",ROUND(MAX(C8-D8,0),2))</f>
+      <c r="F8" s="15" t="n">
+        <f aca="false">IF(C8="","",IF(R8=TRUE(),0,ROUND(MAX(C8-D8,0),2)))</f>
         <v>0</v>
       </c>
-      <c r="G8" s="14" t="n">
-        <f aca="false">IF(C8="",IF(D8&gt;0,D8,""),ROUND(MAX(C8,D8),2))</f>
+      <c r="G8" s="15" t="n">
+        <f aca="false">IF(R8=TRUE(),D8,IF(C8="",IF(D8&gt;0,D8,""),ROUND(MAX(C8,D8),2)))</f>
         <v>11547.01</v>
       </c>
-      <c r="H8" s="14" t="n">
-        <f aca="false">IF(C8="",IF(D8+E8&gt;0,ROUND(D8+E8,2),""),ROUND(G8+E8,2))</f>
+      <c r="H8" s="15" t="n">
+        <f aca="false">IF(G8&lt;&gt;"",ROUND(G8+E8,2),IF(D8+E8&gt;0,ROUND(D8+E8,2),""))</f>
         <v>13247.01</v>
       </c>
-      <c r="I8" s="14" t="n">
+      <c r="I8" s="15" t="n">
         <f aca="false">IF(OR(B8="",G8=""),"",ROUND(G8-B8,2))</f>
         <v>297.01</v>
       </c>
-      <c r="J8" s="15" t="n">
+      <c r="J8" s="16" t="n">
         <f aca="false">IF(I8="","",IF(B8=0,"",I8/B8))</f>
         <v>0.0264008888888889</v>
       </c>
-      <c r="K8" s="14" t="n">
+      <c r="K8" s="15" t="n">
         <f aca="false">IF(I8="","",ROUND(B8-G8,2))</f>
         <v>-297.01</v>
       </c>
-      <c r="L8" s="14" t="n">
+      <c r="L8" s="15" t="n">
         <f aca="false">IF(OR(C8="",D8=0),"",ROUND(D8-C8,2))</f>
         <v>742.68</v>
       </c>
-      <c r="M8" s="15" t="n">
+      <c r="M8" s="16" t="n">
         <f aca="false">IF(L8="","",IF(C8=0,"",L8/C8))</f>
         <v>0.0687391073763945</v>
       </c>
@@ -1551,69 +1606,73 @@
         <f aca="false">IF($A8="unallocated","unallocated_cost",IF(C8="","no_cost_source",IF(D8=0,"unbilled",IF(ABS(D8-C8)&lt;=ABS(C8)*$B$3/100,"within_tolerance","exception"))))</f>
         <v>exception</v>
       </c>
-      <c r="O8" s="11" t="str">
+      <c r="O8" s="12" t="str">
         <f aca="false">Inputs!M2</f>
         <v>source_gap</v>
       </c>
-      <c r="P8" s="14" t="n">
+      <c r="P8" s="15" t="n">
         <f aca="false">IF(I8="","",ABS(I8))</f>
         <v>297.01</v>
       </c>
-      <c r="Q8" s="14" t="n">
+      <c r="Q8" s="15" t="n">
         <f aca="false">IF(I8="","",B8)</f>
         <v>11250</v>
       </c>
+      <c r="R8" s="17" t="b">
+        <f aca="false">Inputs!N2</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="str">
+      <c r="A9" s="12" t="str">
         <f aca="false">Inputs!A3</f>
         <v>google</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="14" t="n">
         <f aca="false">IF(Inputs!B3="","",Inputs!B3)</f>
         <v>8500</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <f aca="false">IF(Inputs!D3="","",Inputs!D3)</f>
         <v>8608.79</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <f aca="false">SUMIFS(Inputs!$E$2:$E$4,Inputs!$A$2:$A$4,$A9)</f>
         <v>8637.19</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="14" t="n">
         <f aca="false">SUMIFS(Inputs!$F$2:$F$4,Inputs!$A$2:$A$4,$A9)</f>
         <v>1133.33</v>
       </c>
-      <c r="F9" s="14" t="n">
-        <f aca="false">IF(C9="","",ROUND(MAX(C9-D9,0),2))</f>
+      <c r="F9" s="15" t="n">
+        <f aca="false">IF(C9="","",IF(R9=TRUE(),0,ROUND(MAX(C9-D9,0),2)))</f>
         <v>0</v>
       </c>
-      <c r="G9" s="14" t="n">
-        <f aca="false">IF(C9="",IF(D9&gt;0,D9,""),ROUND(MAX(C9,D9),2))</f>
+      <c r="G9" s="15" t="n">
+        <f aca="false">IF(R9=TRUE(),D9,IF(C9="",IF(D9&gt;0,D9,""),ROUND(MAX(C9,D9),2)))</f>
         <v>8637.19</v>
       </c>
-      <c r="H9" s="14" t="n">
-        <f aca="false">IF(C9="",IF(D9+E9&gt;0,ROUND(D9+E9,2),""),ROUND(G9+E9,2))</f>
+      <c r="H9" s="15" t="n">
+        <f aca="false">IF(G9&lt;&gt;"",ROUND(G9+E9,2),IF(D9+E9&gt;0,ROUND(D9+E9,2),""))</f>
         <v>9770.52</v>
       </c>
-      <c r="I9" s="14" t="n">
+      <c r="I9" s="15" t="n">
         <f aca="false">IF(OR(B9="",G9=""),"",ROUND(G9-B9,2))</f>
         <v>137.19</v>
       </c>
-      <c r="J9" s="15" t="n">
+      <c r="J9" s="16" t="n">
         <f aca="false">IF(I9="","",IF(B9=0,"",I9/B9))</f>
         <v>0.01614</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="K9" s="15" t="n">
         <f aca="false">IF(I9="","",ROUND(B9-G9,2))</f>
         <v>-137.19</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="L9" s="15" t="n">
         <f aca="false">IF(OR(C9="",D9=0),"",ROUND(D9-C9,2))</f>
         <v>28.4</v>
       </c>
-      <c r="M9" s="15" t="n">
+      <c r="M9" s="16" t="n">
         <f aca="false">IF(L9="","",IF(C9=0,"",L9/C9))</f>
         <v>0.00329895374378978</v>
       </c>
@@ -1621,69 +1680,73 @@
         <f aca="false">IF($A9="unallocated","unallocated_cost",IF(C9="","no_cost_source",IF(D9=0,"unbilled",IF(ABS(D9-C9)&lt;=ABS(C9)*$B$3/100,"within_tolerance","exception"))))</f>
         <v>within_tolerance</v>
       </c>
-      <c r="O9" s="11" t="str">
+      <c r="O9" s="12" t="str">
         <f aca="false">Inputs!M3</f>
         <v>complete</v>
       </c>
-      <c r="P9" s="14" t="n">
+      <c r="P9" s="15" t="n">
         <f aca="false">IF(I9="","",ABS(I9))</f>
         <v>137.19</v>
       </c>
-      <c r="Q9" s="14" t="n">
+      <c r="Q9" s="15" t="n">
         <f aca="false">IF(I9="","",B9)</f>
         <v>8500</v>
       </c>
+      <c r="R9" s="17" t="b">
+        <f aca="false">Inputs!N3</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="str">
+      <c r="A10" s="12" t="str">
         <f aca="false">Inputs!A4</f>
         <v>tiktok</v>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="14" t="n">
         <f aca="false">IF(Inputs!B4="","",Inputs!B4)</f>
         <v>1500</v>
       </c>
-      <c r="C10" s="13" t="str">
+      <c r="C10" s="14" t="str">
         <f aca="false">IF(Inputs!D4="","",Inputs!D4)</f>
         <v/>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <f aca="false">SUMIFS(Inputs!$E$2:$E$4,Inputs!$A$2:$A$4,$A10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="14" t="n">
         <f aca="false">SUMIFS(Inputs!$F$2:$F$4,Inputs!$A$2:$A$4,$A10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="14" t="str">
-        <f aca="false">IF(C10="","",ROUND(MAX(C10-D10,0),2))</f>
+      <c r="F10" s="15" t="str">
+        <f aca="false">IF(C10="","",IF(R10=TRUE(),0,ROUND(MAX(C10-D10,0),2)))</f>
         <v/>
       </c>
-      <c r="G10" s="14" t="str">
-        <f aca="false">IF(C10="",IF(D10&gt;0,D10,""),ROUND(MAX(C10,D10),2))</f>
+      <c r="G10" s="15" t="str">
+        <f aca="false">IF(R10=TRUE(),D10,IF(C10="",IF(D10&gt;0,D10,""),ROUND(MAX(C10,D10),2)))</f>
         <v/>
       </c>
-      <c r="H10" s="14" t="str">
-        <f aca="false">IF(C10="",IF(D10+E10&gt;0,ROUND(D10+E10,2),""),ROUND(G10+E10,2))</f>
+      <c r="H10" s="15" t="str">
+        <f aca="false">IF(G10&lt;&gt;"",ROUND(G10+E10,2),IF(D10+E10&gt;0,ROUND(D10+E10,2),""))</f>
         <v/>
       </c>
-      <c r="I10" s="14" t="str">
+      <c r="I10" s="15" t="str">
         <f aca="false">IF(OR(B10="",G10=""),"",ROUND(G10-B10,2))</f>
         <v/>
       </c>
-      <c r="J10" s="15" t="str">
+      <c r="J10" s="16" t="str">
         <f aca="false">IF(I10="","",IF(B10=0,"",I10/B10))</f>
         <v/>
       </c>
-      <c r="K10" s="14" t="str">
+      <c r="K10" s="15" t="str">
         <f aca="false">IF(I10="","",ROUND(B10-G10,2))</f>
         <v/>
       </c>
-      <c r="L10" s="14" t="str">
+      <c r="L10" s="15" t="str">
         <f aca="false">IF(OR(C10="",D10=0),"",ROUND(D10-C10,2))</f>
         <v/>
       </c>
-      <c r="M10" s="15" t="str">
+      <c r="M10" s="16" t="str">
         <f aca="false">IF(L10="","",IF(C10=0,"",L10/C10))</f>
         <v/>
       </c>
@@ -1691,64 +1754,68 @@
         <f aca="false">IF($A10="unallocated","unallocated_cost",IF(C10="","no_cost_source",IF(D10=0,"unbilled",IF(ABS(D10-C10)&lt;=ABS(C10)*$B$3/100,"within_tolerance","exception"))))</f>
         <v>no_cost_source</v>
       </c>
-      <c r="O10" s="11" t="str">
+      <c r="O10" s="12" t="str">
         <f aca="false">Inputs!M4</f>
         <v>no_cost_source</v>
       </c>
-      <c r="P10" s="14" t="str">
+      <c r="P10" s="15" t="str">
         <f aca="false">IF(I10="","",ABS(I10))</f>
         <v/>
       </c>
-      <c r="Q10" s="14" t="str">
+      <c r="Q10" s="15" t="str">
         <f aca="false">IF(I10="","",B10)</f>
         <v/>
       </c>
+      <c r="R10" s="17" t="b">
+        <f aca="false">Inputs!N4</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B11" s="16" t="n">
+        <v>84</v>
+      </c>
+      <c r="B11" s="18" t="n">
         <f aca="false">SUM(B8:B10)</f>
         <v>21250</v>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="18" t="n">
         <f aca="false">SUM(C8:C10)</f>
         <v>19413.12</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="18" t="n">
         <f aca="false">SUM(D8:D10)</f>
         <v>20184.2</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="18" t="n">
         <f aca="false">SUM(E8:E10)</f>
         <v>2833.33</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="18" t="n">
         <f aca="false">SUM(F8:F10)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="18" t="n">
         <f aca="false">SUM(G8:G10)</f>
         <v>20184.2</v>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="18" t="n">
         <f aca="false">SUM(H8:H10)</f>
         <v>23017.53</v>
       </c>
-      <c r="I11" s="16" t="n">
+      <c r="I11" s="18" t="n">
         <f aca="false">SUM(I8:I10)</f>
         <v>434.2</v>
       </c>
-      <c r="J11" s="17" t="n">
+      <c r="J11" s="19" t="n">
         <f aca="false">IF(Q11=0,"",I11/Q11)</f>
         <v>0.0219848101265823</v>
       </c>
-      <c r="K11" s="16" t="n">
+      <c r="K11" s="18" t="n">
         <f aca="false">SUM(K8:K10)</f>
         <v>-434.2</v>
       </c>
-      <c r="L11" s="16" t="n">
+      <c r="L11" s="18" t="n">
         <f aca="false">SUM(L8:L10)</f>
         <v>771.08</v>
       </c>
@@ -1756,10 +1823,11 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
-      <c r="Q11" s="16" t="n">
+      <c r="Q11" s="18" t="n">
         <f aca="false">SUM(Q8:Q10)</f>
         <v>19750</v>
       </c>
+      <c r="R11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
@@ -1779,10 +1847,11 @@
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>81</v>
+      <c r="A13" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1800,6 +1869,7 @@
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1826,206 +1896,206 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="18" t="b">
+        <v>88</v>
+      </c>
+      <c r="B2" s="20" t="b">
         <f aca="false">ROUND(Month_End!B11-SUM(Inputs!B2:B4),2)=0</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B3" s="18" t="b">
+        <v>89</v>
+      </c>
+      <c r="B3" s="20" t="b">
         <f aca="false">ROUND(Month_End!C11-SUM(Inputs!D2:D4),2)=0</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="18" t="b">
+        <v>90</v>
+      </c>
+      <c r="B4" s="20" t="b">
         <f aca="false">ROUND(Month_End!D11-SUM(Inputs!E2:E4),2)=0</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="18" t="b">
+        <v>91</v>
+      </c>
+      <c r="B5" s="20" t="b">
         <f aca="false">ROUND(Month_End!E11-SUM(Inputs!F2:F4),2)=0</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="18" t="b">
+        <v>92</v>
+      </c>
+      <c r="B6" s="20" t="b">
         <f aca="false">IF(AND(Month_End!F8="",Inputs!G2=""),TRUE(),IF(OR(Month_End!F8="",Inputs!G2=""),FALSE(),ROUND(Month_End!F8-Inputs!G2,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B7" s="18" t="b">
+        <v>93</v>
+      </c>
+      <c r="B7" s="20" t="b">
         <f aca="false">IF(AND(Month_End!G8="",Inputs!H2=""),TRUE(),IF(OR(Month_End!G8="",Inputs!H2=""),FALSE(),ROUND(Month_End!G8-Inputs!H2,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="18" t="b">
+        <v>94</v>
+      </c>
+      <c r="B8" s="20" t="b">
         <f aca="false">IF(AND(Month_End!H8="",Inputs!I2=""),TRUE(),IF(OR(Month_End!H8="",Inputs!I2=""),FALSE(),ROUND(Month_End!H8-Inputs!I2,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="18" t="b">
+        <v>95</v>
+      </c>
+      <c r="B9" s="20" t="b">
         <f aca="false">IF(AND(Month_End!I8="",Inputs!J2=""),TRUE(),IF(OR(Month_End!I8="",Inputs!J2=""),FALSE(),ROUND(Month_End!I8-Inputs!J2,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" s="18" t="b">
+        <v>96</v>
+      </c>
+      <c r="B10" s="20" t="b">
         <f aca="false">IF(AND(Month_End!L8="",Inputs!K2=""),TRUE(),IF(OR(Month_End!L8="",Inputs!K2=""),FALSE(),ROUND(Month_End!L8-Inputs!K2,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B11" s="18" t="b">
+        <v>97</v>
+      </c>
+      <c r="B11" s="20" t="b">
         <f aca="false">Month_End!N8=Inputs!L2</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B12" s="18" t="b">
+        <v>98</v>
+      </c>
+      <c r="B12" s="20" t="b">
         <f aca="false">IF(AND(Month_End!F9="",Inputs!G3=""),TRUE(),IF(OR(Month_End!F9="",Inputs!G3=""),FALSE(),ROUND(Month_End!F9-Inputs!G3,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B13" s="18" t="b">
+        <v>99</v>
+      </c>
+      <c r="B13" s="20" t="b">
         <f aca="false">IF(AND(Month_End!G9="",Inputs!H3=""),TRUE(),IF(OR(Month_End!G9="",Inputs!H3=""),FALSE(),ROUND(Month_End!G9-Inputs!H3,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="18" t="b">
+        <v>100</v>
+      </c>
+      <c r="B14" s="20" t="b">
         <f aca="false">IF(AND(Month_End!H9="",Inputs!I3=""),TRUE(),IF(OR(Month_End!H9="",Inputs!I3=""),FALSE(),ROUND(Month_End!H9-Inputs!I3,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="18" t="b">
+        <v>101</v>
+      </c>
+      <c r="B15" s="20" t="b">
         <f aca="false">IF(AND(Month_End!I9="",Inputs!J3=""),TRUE(),IF(OR(Month_End!I9="",Inputs!J3=""),FALSE(),ROUND(Month_End!I9-Inputs!J3,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" s="18" t="b">
+        <v>102</v>
+      </c>
+      <c r="B16" s="20" t="b">
         <f aca="false">IF(AND(Month_End!L9="",Inputs!K3=""),TRUE(),IF(OR(Month_End!L9="",Inputs!K3=""),FALSE(),ROUND(Month_End!L9-Inputs!K3,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B17" s="18" t="b">
+        <v>103</v>
+      </c>
+      <c r="B17" s="20" t="b">
         <f aca="false">Month_End!N9=Inputs!L3</f>
         <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B18" s="18" t="b">
+        <v>104</v>
+      </c>
+      <c r="B18" s="20" t="b">
         <f aca="false">IF(AND(Month_End!F10="",Inputs!G4=""),TRUE(),IF(OR(Month_End!F10="",Inputs!G4=""),FALSE(),ROUND(Month_End!F10-Inputs!G4,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B19" s="18" t="b">
+        <v>105</v>
+      </c>
+      <c r="B19" s="20" t="b">
         <f aca="false">IF(AND(Month_End!G10="",Inputs!H4=""),TRUE(),IF(OR(Month_End!G10="",Inputs!H4=""),FALSE(),ROUND(Month_End!G10-Inputs!H4,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B20" s="18" t="b">
+        <v>106</v>
+      </c>
+      <c r="B20" s="20" t="b">
         <f aca="false">IF(AND(Month_End!H10="",Inputs!I4=""),TRUE(),IF(OR(Month_End!H10="",Inputs!I4=""),FALSE(),ROUND(Month_End!H10-Inputs!I4,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="18" t="b">
+        <v>107</v>
+      </c>
+      <c r="B21" s="20" t="b">
         <f aca="false">IF(AND(Month_End!I10="",Inputs!J4=""),TRUE(),IF(OR(Month_End!I10="",Inputs!J4=""),FALSE(),ROUND(Month_End!I10-Inputs!J4,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B22" s="18" t="b">
+        <v>108</v>
+      </c>
+      <c r="B22" s="20" t="b">
         <f aca="false">IF(AND(Month_End!L10="",Inputs!K4=""),TRUE(),IF(OR(Month_End!L10="",Inputs!K4=""),FALSE(),ROUND(Month_End!L10-Inputs!K4,2)=0))</f>
         <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B23" s="18" t="b">
+        <v>109</v>
+      </c>
+      <c r="B23" s="20" t="b">
         <f aca="false">Month_End!N10=Inputs!L4</f>
         <v>1</v>
       </c>
@@ -2036,16 +2106,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B25" s="19" t="b">
+        <v>110</v>
+      </c>
+      <c r="B25" s="21" t="b">
         <f aca="false">AND(B2:B23)</f>
         <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
-        <v>107</v>
+      <c r="A26" s="10" t="s">
+        <v>111</v>
       </c>
       <c r="B26" s="2"/>
     </row>
@@ -2073,38 +2143,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="str">
+      <c r="A3" s="22" t="str">
         <f aca="false">"These figures use SYNTHETIC Finance inputs (invented budgets and invoices) and are for demonstration only."</f>
         <v>These figures use SYNTHETIC Finance inputs (invented budgets and invoices) and are for demonstration only.</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="str">
+      <c r="A4" s="22" t="str">
         <f aca="false">IF(COUNT(Month_End!$P$8:$P$10)=0,"No channel has both a media budget and known spend this month.","The largest budget variance in "&amp;Month_End!$B$4&amp;" is "&amp;SUBSTITUTE(PROPER(INDEX(Month_End!$A$8:$A$10,MATCH(MAX(Month_End!$P$8:$P$10),Month_End!$P$8:$P$10,0))),"Tiktok","TikTok")&amp;" at £"&amp;TEXT(ABS(INDEX(Month_End!$I$8:$I$10,MATCH(MAX(Month_End!$P$8:$P$10),Month_End!$P$8:$P$10,0))),"#,##0")&amp;" ("&amp;TEXT(ABS(INDEX(Month_End!$J$8:$J$10,MATCH(MAX(Month_End!$P$8:$P$10),Month_End!$P$8:$P$10,0))),"0.0%")&amp;"), "&amp;IF(INDEX(Month_End!$I$8:$I$10,MATCH(MAX(Month_End!$P$8:$P$10),Month_End!$P$8:$P$10,0))&gt;0,"an overspend","an underspend")&amp;" against its media budget.")</f>
         <v>The largest budget variance in 2025-03 is Meta at £297 (2.6%), an overspend against its media budget.</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="str">
+      <c r="A5" s="22" t="str">
         <f aca="false">IF(COUNTIF(Month_End!$N$8:$N$10,"no_cost_source")=0,"",SUBSTITUTE(PROPER(INDEX(Month_End!$A$8:$A$10,MATCH("no_cost_source",Month_End!$N$8:$N$10,0))),"Tiktok","TikTok")&amp;" has an approved budget of £"&amp;TEXT(INDEX(Month_End!$B$8:$B$10,MATCH("no_cost_source",Month_End!$N$8:$N$10,0)),"#,##0")&amp;" but no cost source, so its spend and variance are unknown (left blank), not zero.")</f>
         <v>TikTok has an approved budget of £1,500 but no cost source, so its spend and variance are unknown (left blank), not zero.</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="str">
+      <c r="A6" s="22" t="str">
         <f aca="false">IF(COUNTIF(Month_End!$N$8:$N$10,"exception")&gt;0,"Main risk: the "&amp;SUBSTITUTE(PROPER(INDEX(Month_End!$A$8:$A$10,MATCH("exception",Month_End!$N$8:$N$10,0))),"Tiktok","TikTok")&amp;" invoice differs from delivered spend by "&amp;TEXT(ABS(INDEX(Month_End!$M$8:$M$10,MATCH("exception",Month_End!$N$8:$N$10,0))),"0.0%")&amp;", above the "&amp;TEXT(Month_End!$B$3,"0.0")&amp;"% tolerance."&amp;IF(INDEX(Month_End!$O$8:$O$10,MATCH("exception",Month_End!$N$8:$N$10,0))="source_gap"," The spend extract is missing days for this month, which may explain the gap.",""),IF(COUNTIF(Month_End!$N$8:$N$10,"unbilled")&gt;0,"Main risk: £"&amp;TEXT(SUM(Month_End!$F$8:$F$10),"#,##0")&amp;" of delivered media is not yet invoiced and is carried as an estimated accrual until the invoices arrive.","Main risk: none flagged. Every platform invoice is within the "&amp;TEXT(Month_End!$B$3,"0.0")&amp;"% tolerance."))</f>
         <v>Main risk: the Meta invoice differs from delivered spend by 6.9%, above the 1.0% tolerance. The spend extract is missing days for this month, which may explain the gap.</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="str">
+      <c r="A7" s="22" t="str">
         <f aca="false">IF(COUNTIF(Month_End!$N$8:$N$10,"exception")&gt;0,IF(INDEX(Month_End!$O$8:$O$10,MATCH("exception",Month_End!$N$8:$N$10,0))="source_gap","Recommended action: obtain the missing days of spend from the platform and re-run the reconciliation before querying the invoice.","Recommended action: query the "&amp;SUBSTITUTE(PROPER(INDEX(Month_End!$A$8:$A$10,MATCH("exception",Month_End!$N$8:$N$10,0))),"Tiktok","TikTok")&amp;" invoice with the platform before approving it for payment."),IF(COUNTIF(Month_End!$N$8:$N$10,"unbilled")&gt;0,"Recommended action: post the £"&amp;TEXT(SUM(Month_End!$F$8:$F$10),"#,##0")&amp;" accrual and replace it with the actual invoices when they arrive early next month.","Recommended action: none beyond normal review."))&amp;IF(COUNTIF(Month_End!$N$8:$N$10,"unallocated_cost")&gt;0," Also allocate the £"&amp;TEXT(SUMIFS(Month_End!$H$8:$H$10,Month_End!$N$8:$N$10,"unallocated_cost"),"#,##0")&amp;" of invoiced cost that has no channel.","")</f>
         <v>Recommended action: obtain the missing days of spend from the platform and re-run the reconciliation before querying the invoice.</v>
       </c>
@@ -2113,8 +2183,8 @@
       <c r="A8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>109</v>
+      <c r="A9" s="10" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>